<commit_message>
data: sync Dades3 MasterFiles + afegir registre manteniment
- Noves SEQs: 087, 237, 240, 287-293 (incl. SEQ_CAL)
- Renames _CAL: 107, 108, 128, 129, 152, 153, 156, 205, 206
- MasterFiles actualitzats (delays, volums)
- Registre manteniment HPLC-DAD-TOC.xlsx afegit
- .gitignore: exclou RAWDATA, backups MasterFile, binaris orfes

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dades3/077B_SEQ_BP/077B_MasterFile.xlsx
+++ b/Dades3/077B_SEQ_BP/077B_MasterFile.xlsx
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5">
@@ -690,7 +690,7 @@
         <v>0.115</v>
       </c>
       <c r="N2" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="O2" t="n">
         <v>0.95</v>
@@ -810,7 +810,7 @@
         <v>0.617</v>
       </c>
       <c r="N4" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
@@ -930,7 +930,7 @@
         <v>0.661</v>
       </c>
       <c r="N6" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="O6" t="n">
         <v>1</v>
@@ -67790,7 +67790,6 @@
       <c r="A2" t="n">
         <v>8</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -67799,7 +67798,6 @@
       <c r="A3" t="n">
         <v>9</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -67808,7 +67806,6 @@
       <c r="A4" t="n">
         <v>10</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -67817,7 +67814,6 @@
       <c r="A5" t="n">
         <v>11</v>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -67826,7 +67822,6 @@
       <c r="A6" t="n">
         <v>12</v>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -67835,7 +67830,6 @@
       <c r="A7" t="n">
         <v>13</v>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -67844,7 +67838,6 @@
       <c r="A8" t="n">
         <v>14</v>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -67853,7 +67846,6 @@
       <c r="A9" t="n">
         <v>15</v>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -67862,7 +67854,6 @@
       <c r="A10" t="n">
         <v>16</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
@@ -67871,7 +67862,6 @@
       <c r="A11" t="n">
         <v>17</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
       </c>
@@ -67880,7 +67870,6 @@
       <c r="A12" t="n">
         <v>18</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>0</v>
       </c>
@@ -67889,7 +67878,6 @@
       <c r="A13" t="n">
         <v>19</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
@@ -67898,7 +67886,6 @@
       <c r="A14" t="n">
         <v>20</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="D14" t="n">
         <v>0</v>
       </c>
@@ -67907,7 +67894,6 @@
       <c r="A15" t="n">
         <v>21</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="D15" t="n">
         <v>0</v>
       </c>
@@ -67916,7 +67902,6 @@
       <c r="A16" t="n">
         <v>22</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="D16" t="n">
         <v>0</v>
       </c>
@@ -67925,7 +67910,6 @@
       <c r="A17" t="n">
         <v>23</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="D17" t="n">
         <v>0</v>
       </c>
@@ -67934,7 +67918,6 @@
       <c r="A18" t="n">
         <v>24</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="D18" t="n">
         <v>0</v>
       </c>
@@ -67943,7 +67926,6 @@
       <c r="A19" t="n">
         <v>25</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="D19" t="n">
         <v>0</v>
       </c>
@@ -67952,7 +67934,6 @@
       <c r="A20" t="n">
         <v>26</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="D20" t="n">
         <v>0</v>
       </c>
@@ -67961,7 +67942,6 @@
       <c r="A21" t="n">
         <v>27</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="D21" t="n">
         <v>0</v>
       </c>
@@ -67970,7 +67950,6 @@
       <c r="A22" t="n">
         <v>28</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="D22" t="n">
         <v>0</v>
       </c>
@@ -67979,7 +67958,6 @@
       <c r="A23" t="n">
         <v>29</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="D23" t="n">
         <v>0</v>
       </c>
@@ -67988,7 +67966,6 @@
       <c r="A24" t="n">
         <v>30</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="D24" t="n">
         <v>0</v>
       </c>
@@ -67997,7 +67974,6 @@
       <c r="A25" t="n">
         <v>31</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="D25" t="n">
         <v>0</v>
       </c>
@@ -68006,7 +67982,6 @@
       <c r="A26" t="n">
         <v>32</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="D26" t="n">
         <v>0</v>
       </c>
@@ -68015,7 +67990,6 @@
       <c r="A27" t="n">
         <v>33</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="D27" t="n">
         <v>0</v>
       </c>
@@ -68024,7 +67998,6 @@
       <c r="A28" t="n">
         <v>34</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="D28" t="n">
         <v>0</v>
       </c>
@@ -68033,7 +68006,6 @@
       <c r="A29" t="n">
         <v>35</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="D29" t="n">
         <v>0</v>
       </c>
@@ -68042,7 +68014,6 @@
       <c r="A30" t="n">
         <v>36</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="D30" t="n">
         <v>0</v>
       </c>
@@ -68051,7 +68022,6 @@
       <c r="A31" t="n">
         <v>37</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="D31" t="n">
         <v>0</v>
       </c>
@@ -68060,7 +68030,6 @@
       <c r="A32" t="n">
         <v>38</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="D32" t="n">
         <v>0</v>
       </c>
@@ -68069,7 +68038,6 @@
       <c r="A33" t="n">
         <v>39</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="D33" t="n">
         <v>0</v>
       </c>
@@ -68078,7 +68046,6 @@
       <c r="A34" t="n">
         <v>40</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="D34" t="n">
         <v>0</v>
       </c>
@@ -68087,7 +68054,6 @@
       <c r="A35" t="n">
         <v>41</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="D35" t="n">
         <v>0</v>
       </c>
@@ -68096,7 +68062,6 @@
       <c r="A36" t="n">
         <v>42</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="D36" t="n">
         <v>0</v>
       </c>
@@ -68105,7 +68070,6 @@
       <c r="A37" t="n">
         <v>43</v>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="D37" t="n">
         <v>0</v>
       </c>
@@ -68114,7 +68078,6 @@
       <c r="A38" t="n">
         <v>44</v>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="D38" t="n">
         <v>0</v>
       </c>
@@ -68123,7 +68086,6 @@
       <c r="A39" t="n">
         <v>45</v>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="D39" t="n">
         <v>0</v>
       </c>
@@ -68132,7 +68094,6 @@
       <c r="A40" t="n">
         <v>46</v>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="D40" t="n">
         <v>0</v>
       </c>
@@ -68141,7 +68102,6 @@
       <c r="A41" t="n">
         <v>47</v>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="D41" t="n">
         <v>0</v>
       </c>
@@ -68150,7 +68110,6 @@
       <c r="A42" t="n">
         <v>48</v>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="D42" t="n">
         <v>0</v>
       </c>
@@ -68159,7 +68118,6 @@
       <c r="A43" t="n">
         <v>49</v>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="D43" t="n">
         <v>0</v>
       </c>
@@ -68168,7 +68126,6 @@
       <c r="A44" t="n">
         <v>50</v>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="D44" t="n">
         <v>0</v>
       </c>
@@ -68177,7 +68134,6 @@
       <c r="A45" t="n">
         <v>51</v>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="D45" t="n">
         <v>0</v>
       </c>
@@ -68186,7 +68142,6 @@
       <c r="A46" t="n">
         <v>52</v>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="D46" t="n">
         <v>0</v>
       </c>
@@ -68195,7 +68150,6 @@
       <c r="A47" t="n">
         <v>53</v>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="D47" t="n">
         <v>0</v>
       </c>
@@ -68204,7 +68158,6 @@
       <c r="A48" t="n">
         <v>54</v>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="D48" t="n">
         <v>0</v>
       </c>
@@ -68213,7 +68166,6 @@
       <c r="A49" t="n">
         <v>55</v>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="D49" t="n">
         <v>0</v>
       </c>
@@ -68222,7 +68174,6 @@
       <c r="A50" t="n">
         <v>56</v>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="D50" t="n">
         <v>0</v>
       </c>
@@ -68231,7 +68182,6 @@
       <c r="A51" t="n">
         <v>57</v>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="D51" t="n">
         <v>0</v>
       </c>
@@ -68240,7 +68190,6 @@
       <c r="A52" t="n">
         <v>58</v>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="D52" t="n">
         <v>0</v>
       </c>
@@ -68249,7 +68198,6 @@
       <c r="A53" t="n">
         <v>59</v>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="D53" t="n">
         <v>0</v>
       </c>
@@ -68258,7 +68206,6 @@
       <c r="A54" t="n">
         <v>60</v>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="D54" t="n">
         <v>0</v>
       </c>
@@ -68267,7 +68214,6 @@
       <c r="A55" t="n">
         <v>61</v>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="D55" t="n">
         <v>0</v>
       </c>
@@ -68276,7 +68222,6 @@
       <c r="A56" t="n">
         <v>62</v>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="D56" t="n">
         <v>0</v>
       </c>
@@ -68285,7 +68230,6 @@
       <c r="A57" t="n">
         <v>63</v>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="D57" t="n">
         <v>0</v>
       </c>
@@ -68294,7 +68238,6 @@
       <c r="A58" t="n">
         <v>64</v>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="D58" t="n">
         <v>0</v>
       </c>
@@ -68303,7 +68246,6 @@
       <c r="A59" t="n">
         <v>65</v>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="D59" t="n">
         <v>0</v>
       </c>
@@ -68312,7 +68254,6 @@
       <c r="A60" t="n">
         <v>66</v>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="D60" t="n">
         <v>0</v>
       </c>
@@ -68321,7 +68262,6 @@
       <c r="A61" t="n">
         <v>67</v>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="D61" t="n">
         <v>0</v>
       </c>
@@ -68330,7 +68270,6 @@
       <c r="A62" t="n">
         <v>68</v>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="D62" t="n">
         <v>0</v>
       </c>
@@ -68339,7 +68278,6 @@
       <c r="A63" t="n">
         <v>69</v>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="D63" t="n">
         <v>0</v>
       </c>
@@ -68348,7 +68286,6 @@
       <c r="A64" t="n">
         <v>70</v>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="D64" t="n">
         <v>0</v>
       </c>
@@ -68357,7 +68294,6 @@
       <c r="A65" t="n">
         <v>71</v>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="D65" t="n">
         <v>0</v>
       </c>
@@ -68366,7 +68302,6 @@
       <c r="A66" t="n">
         <v>72</v>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="D66" t="n">
         <v>0</v>
       </c>
@@ -68375,7 +68310,6 @@
       <c r="A67" t="n">
         <v>73</v>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="D67" t="n">
         <v>0</v>
       </c>
@@ -68384,7 +68318,6 @@
       <c r="A68" t="n">
         <v>74</v>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="D68" t="n">
         <v>0</v>
       </c>
@@ -68393,7 +68326,6 @@
       <c r="A69" t="n">
         <v>75</v>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="D69" t="n">
         <v>0</v>
       </c>
@@ -68402,7 +68334,6 @@
       <c r="A70" t="n">
         <v>76</v>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="D70" t="n">
         <v>0</v>
       </c>
@@ -68411,7 +68342,6 @@
       <c r="A71" t="n">
         <v>77</v>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="D71" t="n">
         <v>0</v>
       </c>
@@ -68420,7 +68350,6 @@
       <c r="A72" t="n">
         <v>78</v>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="D72" t="n">
         <v>0</v>
       </c>
@@ -68429,7 +68358,6 @@
       <c r="A73" t="n">
         <v>79</v>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="D73" t="n">
         <v>0</v>
       </c>
@@ -68438,7 +68366,6 @@
       <c r="A74" t="n">
         <v>80</v>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="D74" t="n">
         <v>0</v>
       </c>
@@ -68447,7 +68374,6 @@
       <c r="A75" t="n">
         <v>81</v>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="D75" t="n">
         <v>0</v>
       </c>
@@ -68456,7 +68382,6 @@
       <c r="A76" t="n">
         <v>82</v>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="D76" t="n">
         <v>0</v>
       </c>
@@ -68465,7 +68390,6 @@
       <c r="A77" t="n">
         <v>83</v>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="D77" t="n">
         <v>0</v>
       </c>
@@ -68474,7 +68398,6 @@
       <c r="A78" t="n">
         <v>84</v>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="D78" t="n">
         <v>0</v>
       </c>
@@ -68483,7 +68406,6 @@
       <c r="A79" t="n">
         <v>85</v>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="D79" t="n">
         <v>0</v>
       </c>
@@ -68492,7 +68414,6 @@
       <c r="A80" t="n">
         <v>86</v>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="D80" t="n">
         <v>0</v>
       </c>
@@ -68501,7 +68422,6 @@
       <c r="A81" t="n">
         <v>87</v>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="D81" t="n">
         <v>0</v>
       </c>
@@ -68510,7 +68430,6 @@
       <c r="A82" t="n">
         <v>88</v>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="D82" t="n">
         <v>0</v>
       </c>
@@ -68519,7 +68438,6 @@
       <c r="A83" t="n">
         <v>89</v>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="D83" t="n">
         <v>0</v>
       </c>
@@ -68528,7 +68446,6 @@
       <c r="A84" t="n">
         <v>90</v>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="D84" t="n">
         <v>0</v>
       </c>
@@ -68537,7 +68454,6 @@
       <c r="A85" t="n">
         <v>91</v>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="D85" t="n">
         <v>0</v>
       </c>
@@ -68546,7 +68462,6 @@
       <c r="A86" t="n">
         <v>92</v>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="D86" t="n">
         <v>0</v>
       </c>
@@ -68555,7 +68470,6 @@
       <c r="A87" t="n">
         <v>93</v>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="D87" t="n">
         <v>0</v>
       </c>
@@ -68564,7 +68478,6 @@
       <c r="A88" t="n">
         <v>94</v>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="D88" t="n">
         <v>0</v>
       </c>
@@ -68573,7 +68486,6 @@
       <c r="A89" t="n">
         <v>95</v>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="D89" t="n">
         <v>0</v>
       </c>
@@ -68582,7 +68494,6 @@
       <c r="A90" t="n">
         <v>96</v>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="D90" t="n">
         <v>0</v>
       </c>
@@ -68591,7 +68502,6 @@
       <c r="A91" t="n">
         <v>97</v>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="D91" t="n">
         <v>0</v>
       </c>
@@ -68600,7 +68510,6 @@
       <c r="A92" t="n">
         <v>98</v>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="D92" t="n">
         <v>0</v>
       </c>
@@ -68609,7 +68518,6 @@
       <c r="A93" t="n">
         <v>99</v>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="D93" t="n">
         <v>0</v>
       </c>
@@ -68618,7 +68526,6 @@
       <c r="A94" t="n">
         <v>100</v>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="D94" t="n">
         <v>0</v>
       </c>
@@ -68627,7 +68534,6 @@
       <c r="A95" t="n">
         <v>101</v>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="D95" t="n">
         <v>0</v>
       </c>
@@ -68636,7 +68542,6 @@
       <c r="A96" t="n">
         <v>102</v>
       </c>
-      <c r="B96" t="inlineStr"/>
       <c r="D96" t="n">
         <v>0</v>
       </c>
@@ -68645,7 +68550,6 @@
       <c r="A97" t="n">
         <v>103</v>
       </c>
-      <c r="B97" t="inlineStr"/>
       <c r="D97" t="n">
         <v>0</v>
       </c>
@@ -68654,7 +68558,6 @@
       <c r="A98" t="n">
         <v>104</v>
       </c>
-      <c r="B98" t="inlineStr"/>
       <c r="D98" t="n">
         <v>0</v>
       </c>
@@ -68663,7 +68566,6 @@
       <c r="A99" t="n">
         <v>105</v>
       </c>
-      <c r="B99" t="inlineStr"/>
       <c r="D99" t="n">
         <v>0</v>
       </c>
@@ -68672,7 +68574,6 @@
       <c r="A100" t="n">
         <v>106</v>
       </c>
-      <c r="B100" t="inlineStr"/>
       <c r="D100" t="n">
         <v>0</v>
       </c>
@@ -68681,7 +68582,6 @@
       <c r="A101" t="n">
         <v>107</v>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="D101" t="n">
         <v>0</v>
       </c>
@@ -68690,7 +68590,6 @@
       <c r="A102" t="n">
         <v>108</v>
       </c>
-      <c r="B102" t="inlineStr"/>
       <c r="D102" t="n">
         <v>0</v>
       </c>
@@ -68699,7 +68598,6 @@
       <c r="A103" t="n">
         <v>109</v>
       </c>
-      <c r="B103" t="inlineStr"/>
       <c r="D103" t="n">
         <v>0</v>
       </c>
@@ -68708,7 +68606,6 @@
       <c r="A104" t="n">
         <v>110</v>
       </c>
-      <c r="B104" t="inlineStr"/>
       <c r="D104" t="n">
         <v>0</v>
       </c>
@@ -68717,7 +68614,6 @@
       <c r="A105" t="n">
         <v>111</v>
       </c>
-      <c r="B105" t="inlineStr"/>
       <c r="D105" t="n">
         <v>0</v>
       </c>
@@ -68726,7 +68622,6 @@
       <c r="A106" t="n">
         <v>112</v>
       </c>
-      <c r="B106" t="inlineStr"/>
       <c r="D106" t="n">
         <v>0</v>
       </c>
@@ -68735,7 +68630,6 @@
       <c r="A107" t="n">
         <v>113</v>
       </c>
-      <c r="B107" t="inlineStr"/>
       <c r="D107" t="n">
         <v>0</v>
       </c>
@@ -68744,7 +68638,6 @@
       <c r="A108" t="n">
         <v>114</v>
       </c>
-      <c r="B108" t="inlineStr"/>
       <c r="D108" t="n">
         <v>0</v>
       </c>
@@ -68753,7 +68646,6 @@
       <c r="A109" t="n">
         <v>115</v>
       </c>
-      <c r="B109" t="inlineStr"/>
       <c r="D109" t="n">
         <v>0</v>
       </c>
@@ -68762,7 +68654,6 @@
       <c r="A110" t="n">
         <v>116</v>
       </c>
-      <c r="B110" t="inlineStr"/>
       <c r="D110" t="n">
         <v>0</v>
       </c>
@@ -68771,7 +68662,6 @@
       <c r="A111" t="n">
         <v>117</v>
       </c>
-      <c r="B111" t="inlineStr"/>
       <c r="D111" t="n">
         <v>0</v>
       </c>
@@ -68780,7 +68670,6 @@
       <c r="A112" t="n">
         <v>118</v>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="D112" t="n">
         <v>0</v>
       </c>
@@ -68789,7 +68678,6 @@
       <c r="A113" t="n">
         <v>119</v>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="D113" t="n">
         <v>0</v>
       </c>
@@ -68798,7 +68686,6 @@
       <c r="A114" t="n">
         <v>120</v>
       </c>
-      <c r="B114" t="inlineStr"/>
       <c r="D114" t="n">
         <v>0</v>
       </c>
@@ -68807,7 +68694,6 @@
       <c r="A115" t="n">
         <v>121</v>
       </c>
-      <c r="B115" t="inlineStr"/>
       <c r="D115" t="n">
         <v>0</v>
       </c>
@@ -68816,7 +68702,6 @@
       <c r="A116" t="n">
         <v>122</v>
       </c>
-      <c r="B116" t="inlineStr"/>
       <c r="D116" t="n">
         <v>0</v>
       </c>
@@ -68825,7 +68710,6 @@
       <c r="A117" t="n">
         <v>123</v>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="D117" t="n">
         <v>0</v>
       </c>
@@ -68834,7 +68718,6 @@
       <c r="A118" t="n">
         <v>124</v>
       </c>
-      <c r="B118" t="inlineStr"/>
       <c r="D118" t="n">
         <v>0</v>
       </c>
@@ -68843,7 +68726,6 @@
       <c r="A119" t="n">
         <v>125</v>
       </c>
-      <c r="B119" t="inlineStr"/>
       <c r="D119" t="n">
         <v>0</v>
       </c>
@@ -68852,7 +68734,6 @@
       <c r="A120" t="n">
         <v>126</v>
       </c>
-      <c r="B120" t="inlineStr"/>
       <c r="D120" t="n">
         <v>0</v>
       </c>
@@ -68861,7 +68742,6 @@
       <c r="A121" t="n">
         <v>127</v>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="D121" t="n">
         <v>0</v>
       </c>
@@ -68870,7 +68750,6 @@
       <c r="A122" t="n">
         <v>128</v>
       </c>
-      <c r="B122" t="inlineStr"/>
       <c r="D122" t="n">
         <v>0</v>
       </c>
@@ -68879,7 +68758,6 @@
       <c r="A123" t="n">
         <v>129</v>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="D123" t="n">
         <v>0</v>
       </c>
@@ -68888,7 +68766,6 @@
       <c r="A124" t="n">
         <v>130</v>
       </c>
-      <c r="B124" t="inlineStr"/>
       <c r="D124" t="n">
         <v>0</v>
       </c>
@@ -68897,7 +68774,6 @@
       <c r="A125" t="n">
         <v>131</v>
       </c>
-      <c r="B125" t="inlineStr"/>
       <c r="D125" t="n">
         <v>0</v>
       </c>
@@ -68906,7 +68782,6 @@
       <c r="A126" t="n">
         <v>132</v>
       </c>
-      <c r="B126" t="inlineStr"/>
       <c r="D126" t="n">
         <v>0</v>
       </c>
@@ -68915,7 +68790,6 @@
       <c r="A127" t="n">
         <v>133</v>
       </c>
-      <c r="B127" t="inlineStr"/>
       <c r="D127" t="n">
         <v>0</v>
       </c>
@@ -68924,7 +68798,6 @@
       <c r="A128" t="n">
         <v>134</v>
       </c>
-      <c r="B128" t="inlineStr"/>
       <c r="D128" t="n">
         <v>0</v>
       </c>
@@ -68933,7 +68806,6 @@
       <c r="A129" t="n">
         <v>135</v>
       </c>
-      <c r="B129" t="inlineStr"/>
       <c r="D129" t="n">
         <v>0</v>
       </c>
@@ -68942,7 +68814,6 @@
       <c r="A130" t="n">
         <v>136</v>
       </c>
-      <c r="B130" t="inlineStr"/>
       <c r="D130" t="n">
         <v>0</v>
       </c>
@@ -68951,7 +68822,6 @@
       <c r="A131" t="n">
         <v>137</v>
       </c>
-      <c r="B131" t="inlineStr"/>
       <c r="D131" t="n">
         <v>0</v>
       </c>
@@ -68960,7 +68830,6 @@
       <c r="A132" t="n">
         <v>138</v>
       </c>
-      <c r="B132" t="inlineStr"/>
       <c r="D132" t="n">
         <v>0</v>
       </c>
@@ -68969,7 +68838,6 @@
       <c r="A133" t="n">
         <v>139</v>
       </c>
-      <c r="B133" t="inlineStr"/>
       <c r="D133" t="n">
         <v>0</v>
       </c>
@@ -68978,7 +68846,6 @@
       <c r="A134" t="n">
         <v>140</v>
       </c>
-      <c r="B134" t="inlineStr"/>
       <c r="D134" t="n">
         <v>0</v>
       </c>
@@ -68987,7 +68854,6 @@
       <c r="A135" t="n">
         <v>141</v>
       </c>
-      <c r="B135" t="inlineStr"/>
       <c r="D135" t="n">
         <v>0</v>
       </c>
@@ -68996,7 +68862,6 @@
       <c r="A136" t="n">
         <v>142</v>
       </c>
-      <c r="B136" t="inlineStr"/>
       <c r="D136" t="n">
         <v>0</v>
       </c>
@@ -69005,7 +68870,6 @@
       <c r="A137" t="n">
         <v>143</v>
       </c>
-      <c r="B137" t="inlineStr"/>
       <c r="D137" t="n">
         <v>0</v>
       </c>
@@ -69014,7 +68878,6 @@
       <c r="A138" t="n">
         <v>144</v>
       </c>
-      <c r="B138" t="inlineStr"/>
       <c r="D138" t="n">
         <v>0</v>
       </c>
@@ -69023,7 +68886,6 @@
       <c r="A139" t="n">
         <v>145</v>
       </c>
-      <c r="B139" t="inlineStr"/>
       <c r="D139" t="n">
         <v>0</v>
       </c>
@@ -69032,7 +68894,6 @@
       <c r="A140" t="n">
         <v>146</v>
       </c>
-      <c r="B140" t="inlineStr"/>
       <c r="D140" t="n">
         <v>0</v>
       </c>
@@ -69041,7 +68902,6 @@
       <c r="A141" t="n">
         <v>147</v>
       </c>
-      <c r="B141" t="inlineStr"/>
       <c r="D141" t="n">
         <v>0</v>
       </c>
@@ -69050,7 +68910,6 @@
       <c r="A142" t="n">
         <v>148</v>
       </c>
-      <c r="B142" t="inlineStr"/>
       <c r="D142" t="n">
         <v>0</v>
       </c>
@@ -69059,7 +68918,6 @@
       <c r="A143" t="n">
         <v>149</v>
       </c>
-      <c r="B143" t="inlineStr"/>
       <c r="D143" t="n">
         <v>0</v>
       </c>
@@ -69068,7 +68926,6 @@
       <c r="A144" t="n">
         <v>150</v>
       </c>
-      <c r="B144" t="inlineStr"/>
       <c r="D144" t="n">
         <v>0</v>
       </c>
@@ -69077,7 +68934,6 @@
       <c r="A145" t="n">
         <v>151</v>
       </c>
-      <c r="B145" t="inlineStr"/>
       <c r="D145" t="n">
         <v>0</v>
       </c>
@@ -69086,7 +68942,6 @@
       <c r="A146" t="n">
         <v>152</v>
       </c>
-      <c r="B146" t="inlineStr"/>
       <c r="D146" t="n">
         <v>0</v>
       </c>
@@ -69095,7 +68950,6 @@
       <c r="A147" t="n">
         <v>153</v>
       </c>
-      <c r="B147" t="inlineStr"/>
       <c r="D147" t="n">
         <v>0</v>
       </c>
@@ -69104,7 +68958,6 @@
       <c r="A148" t="n">
         <v>154</v>
       </c>
-      <c r="B148" t="inlineStr"/>
       <c r="D148" t="n">
         <v>0</v>
       </c>
@@ -69113,7 +68966,6 @@
       <c r="A149" t="n">
         <v>155</v>
       </c>
-      <c r="B149" t="inlineStr"/>
       <c r="D149" t="n">
         <v>0</v>
       </c>
@@ -69122,7 +68974,6 @@
       <c r="A150" t="n">
         <v>156</v>
       </c>
-      <c r="B150" t="inlineStr"/>
       <c r="D150" t="n">
         <v>0</v>
       </c>
@@ -69131,7 +68982,6 @@
       <c r="A151" t="n">
         <v>157</v>
       </c>
-      <c r="B151" t="inlineStr"/>
       <c r="D151" t="n">
         <v>0</v>
       </c>
@@ -69140,7 +68990,6 @@
       <c r="A152" t="n">
         <v>158</v>
       </c>
-      <c r="B152" t="inlineStr"/>
       <c r="D152" t="n">
         <v>0</v>
       </c>
@@ -69149,7 +68998,6 @@
       <c r="A153" t="n">
         <v>159</v>
       </c>
-      <c r="B153" t="inlineStr"/>
       <c r="D153" t="n">
         <v>0</v>
       </c>
@@ -69158,7 +69006,6 @@
       <c r="A154" t="n">
         <v>160</v>
       </c>
-      <c r="B154" t="inlineStr"/>
       <c r="D154" t="n">
         <v>0</v>
       </c>
@@ -69167,7 +69014,6 @@
       <c r="A155" t="n">
         <v>161</v>
       </c>
-      <c r="B155" t="inlineStr"/>
       <c r="D155" t="n">
         <v>0</v>
       </c>
@@ -69176,7 +69022,6 @@
       <c r="A156" t="n">
         <v>162</v>
       </c>
-      <c r="B156" t="inlineStr"/>
       <c r="D156" t="n">
         <v>0</v>
       </c>
@@ -69185,7 +69030,6 @@
       <c r="A157" t="n">
         <v>163</v>
       </c>
-      <c r="B157" t="inlineStr"/>
       <c r="D157" t="n">
         <v>0</v>
       </c>
@@ -69194,7 +69038,6 @@
       <c r="A158" t="n">
         <v>164</v>
       </c>
-      <c r="B158" t="inlineStr"/>
       <c r="D158" t="n">
         <v>0</v>
       </c>
@@ -69203,7 +69046,6 @@
       <c r="A159" t="n">
         <v>165</v>
       </c>
-      <c r="B159" t="inlineStr"/>
       <c r="D159" t="n">
         <v>0</v>
       </c>
@@ -69212,7 +69054,6 @@
       <c r="A160" t="n">
         <v>166</v>
       </c>
-      <c r="B160" t="inlineStr"/>
       <c r="D160" t="n">
         <v>0</v>
       </c>
@@ -69221,7 +69062,6 @@
       <c r="A161" t="n">
         <v>167</v>
       </c>
-      <c r="B161" t="inlineStr"/>
       <c r="D161" t="n">
         <v>0</v>
       </c>
@@ -69230,7 +69070,6 @@
       <c r="A162" t="n">
         <v>168</v>
       </c>
-      <c r="B162" t="inlineStr"/>
       <c r="D162" t="n">
         <v>0</v>
       </c>
@@ -69239,7 +69078,6 @@
       <c r="A163" t="n">
         <v>169</v>
       </c>
-      <c r="B163" t="inlineStr"/>
       <c r="D163" t="n">
         <v>0</v>
       </c>
@@ -69248,7 +69086,6 @@
       <c r="A164" t="n">
         <v>170</v>
       </c>
-      <c r="B164" t="inlineStr"/>
       <c r="D164" t="n">
         <v>0</v>
       </c>
@@ -69257,7 +69094,6 @@
       <c r="A165" t="n">
         <v>171</v>
       </c>
-      <c r="B165" t="inlineStr"/>
       <c r="D165" t="n">
         <v>0</v>
       </c>
@@ -69266,7 +69102,6 @@
       <c r="A166" t="n">
         <v>172</v>
       </c>
-      <c r="B166" t="inlineStr"/>
       <c r="D166" t="n">
         <v>0</v>
       </c>
@@ -69275,7 +69110,6 @@
       <c r="A167" t="n">
         <v>173</v>
       </c>
-      <c r="B167" t="inlineStr"/>
       <c r="D167" t="n">
         <v>0</v>
       </c>
@@ -69284,7 +69118,6 @@
       <c r="A168" t="n">
         <v>174</v>
       </c>
-      <c r="B168" t="inlineStr"/>
       <c r="D168" t="n">
         <v>0</v>
       </c>
@@ -69293,7 +69126,6 @@
       <c r="A169" t="n">
         <v>175</v>
       </c>
-      <c r="B169" t="inlineStr"/>
       <c r="D169" t="n">
         <v>0</v>
       </c>
@@ -69302,7 +69134,6 @@
       <c r="A170" t="n">
         <v>176</v>
       </c>
-      <c r="B170" t="inlineStr"/>
       <c r="D170" t="n">
         <v>0</v>
       </c>
@@ -69311,7 +69142,6 @@
       <c r="A171" t="n">
         <v>177</v>
       </c>
-      <c r="B171" t="inlineStr"/>
       <c r="D171" t="n">
         <v>0</v>
       </c>
@@ -69320,7 +69150,6 @@
       <c r="A172" t="n">
         <v>178</v>
       </c>
-      <c r="B172" t="inlineStr"/>
       <c r="D172" t="n">
         <v>0</v>
       </c>
@@ -69329,7 +69158,6 @@
       <c r="A173" t="n">
         <v>179</v>
       </c>
-      <c r="B173" t="inlineStr"/>
       <c r="D173" t="n">
         <v>0</v>
       </c>
@@ -69338,7 +69166,6 @@
       <c r="A174" t="n">
         <v>180</v>
       </c>
-      <c r="B174" t="inlineStr"/>
       <c r="D174" t="n">
         <v>0</v>
       </c>
@@ -69347,7 +69174,6 @@
       <c r="A175" t="n">
         <v>181</v>
       </c>
-      <c r="B175" t="inlineStr"/>
       <c r="D175" t="n">
         <v>0</v>
       </c>
@@ -69356,7 +69182,6 @@
       <c r="A176" t="n">
         <v>182</v>
       </c>
-      <c r="B176" t="inlineStr"/>
       <c r="D176" t="n">
         <v>0</v>
       </c>
@@ -69365,7 +69190,6 @@
       <c r="A177" t="n">
         <v>183</v>
       </c>
-      <c r="B177" t="inlineStr"/>
       <c r="D177" t="n">
         <v>0</v>
       </c>
@@ -69374,7 +69198,6 @@
       <c r="A178" t="n">
         <v>184</v>
       </c>
-      <c r="B178" t="inlineStr"/>
       <c r="D178" t="n">
         <v>0</v>
       </c>
@@ -69383,7 +69206,6 @@
       <c r="A179" t="n">
         <v>185</v>
       </c>
-      <c r="B179" t="inlineStr"/>
       <c r="D179" t="n">
         <v>0</v>
       </c>
@@ -69392,7 +69214,6 @@
       <c r="A180" t="n">
         <v>186</v>
       </c>
-      <c r="B180" t="inlineStr"/>
       <c r="D180" t="n">
         <v>0</v>
       </c>
@@ -69401,7 +69222,6 @@
       <c r="A181" t="n">
         <v>187</v>
       </c>
-      <c r="B181" t="inlineStr"/>
       <c r="D181" t="n">
         <v>0</v>
       </c>
@@ -69410,7 +69230,6 @@
       <c r="A182" t="n">
         <v>188</v>
       </c>
-      <c r="B182" t="inlineStr"/>
       <c r="D182" t="n">
         <v>0</v>
       </c>
@@ -69419,7 +69238,6 @@
       <c r="A183" t="n">
         <v>189</v>
       </c>
-      <c r="B183" t="inlineStr"/>
       <c r="D183" t="n">
         <v>0</v>
       </c>
@@ -69428,7 +69246,6 @@
       <c r="A184" t="n">
         <v>190</v>
       </c>
-      <c r="B184" t="inlineStr"/>
       <c r="D184" t="n">
         <v>0</v>
       </c>
@@ -69437,7 +69254,6 @@
       <c r="A185" t="n">
         <v>191</v>
       </c>
-      <c r="B185" t="inlineStr"/>
       <c r="D185" t="n">
         <v>0</v>
       </c>
@@ -69446,7 +69262,6 @@
       <c r="A186" t="n">
         <v>192</v>
       </c>
-      <c r="B186" t="inlineStr"/>
       <c r="D186" t="n">
         <v>0</v>
       </c>
@@ -69455,7 +69270,6 @@
       <c r="A187" t="n">
         <v>193</v>
       </c>
-      <c r="B187" t="inlineStr"/>
       <c r="D187" t="n">
         <v>0</v>
       </c>
@@ -69464,7 +69278,6 @@
       <c r="A188" t="n">
         <v>194</v>
       </c>
-      <c r="B188" t="inlineStr"/>
       <c r="D188" t="n">
         <v>0</v>
       </c>
@@ -69473,7 +69286,6 @@
       <c r="A189" t="n">
         <v>195</v>
       </c>
-      <c r="B189" t="inlineStr"/>
       <c r="D189" t="n">
         <v>0</v>
       </c>
@@ -69482,7 +69294,6 @@
       <c r="A190" t="n">
         <v>196</v>
       </c>
-      <c r="B190" t="inlineStr"/>
       <c r="D190" t="n">
         <v>0</v>
       </c>
@@ -69491,7 +69302,6 @@
       <c r="A191" t="n">
         <v>197</v>
       </c>
-      <c r="B191" t="inlineStr"/>
       <c r="D191" t="n">
         <v>0</v>
       </c>
@@ -69500,7 +69310,6 @@
       <c r="A192" t="n">
         <v>198</v>
       </c>
-      <c r="B192" t="inlineStr"/>
       <c r="D192" t="n">
         <v>0</v>
       </c>
@@ -69509,7 +69318,6 @@
       <c r="A193" t="n">
         <v>199</v>
       </c>
-      <c r="B193" t="inlineStr"/>
       <c r="D193" t="n">
         <v>0</v>
       </c>
@@ -69518,7 +69326,6 @@
       <c r="A194" t="n">
         <v>200</v>
       </c>
-      <c r="B194" t="inlineStr"/>
       <c r="D194" t="n">
         <v>0</v>
       </c>
@@ -69527,7 +69334,6 @@
       <c r="A195" t="n">
         <v>201</v>
       </c>
-      <c r="B195" t="inlineStr"/>
       <c r="D195" t="n">
         <v>0</v>
       </c>
@@ -69536,7 +69342,6 @@
       <c r="A196" t="n">
         <v>202</v>
       </c>
-      <c r="B196" t="inlineStr"/>
       <c r="D196" t="n">
         <v>0</v>
       </c>
@@ -69545,7 +69350,6 @@
       <c r="A197" t="n">
         <v>203</v>
       </c>
-      <c r="B197" t="inlineStr"/>
       <c r="D197" t="n">
         <v>0</v>
       </c>
@@ -69554,7 +69358,6 @@
       <c r="A198" t="n">
         <v>204</v>
       </c>
-      <c r="B198" t="inlineStr"/>
       <c r="D198" t="n">
         <v>0</v>
       </c>
@@ -69563,7 +69366,6 @@
       <c r="A199" t="n">
         <v>205</v>
       </c>
-      <c r="B199" t="inlineStr"/>
       <c r="D199" t="n">
         <v>0</v>
       </c>
@@ -69572,7 +69374,6 @@
       <c r="A200" t="n">
         <v>206</v>
       </c>
-      <c r="B200" t="inlineStr"/>
       <c r="D200" t="n">
         <v>0</v>
       </c>
@@ -69581,7 +69382,6 @@
       <c r="A201" t="n">
         <v>207</v>
       </c>
-      <c r="B201" t="inlineStr"/>
       <c r="D201" t="n">
         <v>0</v>
       </c>
@@ -69590,7 +69390,6 @@
       <c r="A202" t="n">
         <v>208</v>
       </c>
-      <c r="B202" t="inlineStr"/>
       <c r="D202" t="n">
         <v>0</v>
       </c>
@@ -69599,7 +69398,6 @@
       <c r="A203" t="n">
         <v>209</v>
       </c>
-      <c r="B203" t="inlineStr"/>
       <c r="D203" t="n">
         <v>0</v>
       </c>

</xml_diff>